<commit_message>
refactor(data): remove internal config revisions
</commit_message>
<xml_diff>
--- a/config/data/ConfigManifest.xlsx
+++ b/config/data/ConfigManifest.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -24,16 +24,68 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F3A4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9EEF5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D6E8F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE5EF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -41,12 +93,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,347 +497,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.7109375" customWidth="1" min="1" max="1"/>
+    <col width="12.7109375" customWidth="1" style="5" min="2" max="2"/>
+    <col width="13.7109375" customWidth="1" style="5" min="3" max="3"/>
+    <col width="16.7109375" customWidth="1" style="5" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>@table</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>ConfigManifest</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>@mode</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>singleton</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>@key</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>@scope</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>@schema</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>857f0dc27c73bc6d</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>2b0b6fe6d3b06bdc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>#name</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>game_version</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>snapshot_date</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>data_revision</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>required_rules_revision</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>sora_cli_version</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>numeric_policy_revision</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>rng_algorithm_revision</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>state_hash_revision</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>replay_format_version</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>coverage_manifest_sha256</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#field</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>game_version</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>snapshot_date</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>data_revision</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>required_rules_revision</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>sora_cli_version</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>numeric_policy_revision</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>rng_algorithm_revision</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>state_hash_revision</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>replay_format_version</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>coverage_manifest_sha256</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#type</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>#scope</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>#input</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>length=1..32</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>length=10..10</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>length=1..80</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>length=1..80</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>length=1..32</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>length=1..80</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>length=1..80</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>length=1..80</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>length=1..80</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>length=64..64</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>#desc</t>
         </is>
       </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -767,42 +687,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>core-combat-v1-phase7-l11</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>core-combat-rules-v1</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
           <t>0.3.0</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>fixed-i64-6dp-v1</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>chacha8-rand-0.10.2-intmap-v1</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>sha256-v5</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>replay-v1</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>e2188c7844d678253c98d569db017dbad7101541cf502aba4c2eb80c0435bf19</t>
         </is>
       </c>
     </row>

</xml_diff>